<commit_message>
Working through more architectural decisions
</commit_message>
<xml_diff>
--- a/portfolio-command-field-inventory.xlsx
+++ b/portfolio-command-field-inventory.xlsx
@@ -27,12 +27,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2955" uniqueCount="900">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2985" uniqueCount="920">
   <si>
     <t xml:space="preserve">Portfolio Command - Master Data Field Inventory</t>
   </si>
   <si>
-    <t xml:space="preserve">Rev 3 - 27 July 2026. All twelve questions and four of six open items closed. Outstanding decisions are tracked on the Decisions &amp; Actions sheet.</t>
+    <t xml:space="preserve">Rev 4 - 28 July 2026. All twelve questions and all six open items closed. Two decisions outstanding with the VC team lead: D-1 and D-6.</t>
   </si>
   <si>
     <t xml:space="preserve">What changed in this revision</t>
@@ -92,7 +92,7 @@
     <t xml:space="preserve">Open</t>
   </si>
   <si>
-    <t xml:space="preserve">Needs a decision from the VC team lead. Cross-referenced to D-1 to D-6 on the Decisions &amp; Actions sheet.</t>
+    <t xml:space="preserve">Outstanding decision. Only D-1 and D-6 remain, both with the VC team lead.</t>
   </si>
   <si>
     <t xml:space="preserve">Field counts (live formulas)</t>
@@ -1169,7 +1169,7 @@
     <t xml:space="preserve">$M run-rate</t>
   </si>
   <si>
-    <t xml:space="preserve">RESOLVED AS FACT (O-5), STILL OPEN AS A DECISION (D-2): Visible supplies the PAST QUARTER'S ACTUAL revenue, not run-rate. Daniel's tile, memo prefill and user guide all label it run-rate. Arithmetic unaffected; the label is wrong. Decision D-2 with the VC team lead.</t>
+    <t xml:space="preserve">RESOLVED (O-5 / D-2): Visible supplies the PAST QUARTER'S ACTUAL revenue. Stored and displayed AS REPORTED - no annualisation. Label moves from run-rate to quarterly revenue in the tile, memo prefill and guide. Note the aggregate figure is ~1/4 of the old run-rate presentation, and same-store QoQ now carries seasonality (phase-2 review).</t>
   </si>
   <si>
     <t xml:space="preserve">burn</t>
@@ -2594,61 +2594,64 @@
     <t xml:space="preserve">D-1</t>
   </si>
   <si>
-    <t xml:space="preserve">VC team lead</t>
+    <t xml:space="preserve">OUTSTANDING</t>
   </si>
   <si>
     <t xml:space="preserve">Confirm the import contract may treat derived fields as advisory, correcting them against the transactions and returning a reconciliation warning.</t>
   </si>
   <si>
-    <t xml:space="preserve">His stated requirement was that the contract stay intact. This is the one place his workflow behaviour changes.</t>
+    <t xml:space="preserve">Still to be walked through with Daniel. His stated requirement was that the contract stay intact; this is the one place his workflow behaviour changes.</t>
   </si>
   <si>
     <t xml:space="preserve">Daniel Armali</t>
   </si>
   <si>
+    <t xml:space="preserve">D-6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Confirm which quarter convention each screen displays, now that fiscal and calendar labels differ.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Still to be walked through with Daniel. Suggested split: fiscal on Reports and board-facing views, calendar on the Portfolio KPI history.</t>
+  </si>
+  <si>
     <t xml:space="preserve">D-2</t>
   </si>
   <si>
-    <t xml:space="preserve">Choose how revenue is presented. Visible supplies quarterly actuals; the prototype labels the figure run-rate.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PRIORITY. His metric and his label, and the only genuine conflict between freezing definitions and changing nothing on screen. Recommended: relabel as quarterly revenue.</t>
+    <t xml:space="preserve">Settled</t>
+  </si>
+  <si>
+    <t xml:space="preserve">How revenue is presented.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DISPLAY AS REPORTED. Visible's quarterly actual stored and shown unchanged, no annualisation. Label moves to quarterly revenue.</t>
   </si>
   <si>
     <t xml:space="preserve">D-3</t>
   </si>
   <si>
-    <t xml:space="preserve">Accept that FMV growth shows two flat quarters per year, labelled as carry-forward.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Visible change in behaviour on a dashboard tile he designed. Cadence is not changing, so the platform labels it.</t>
+    <t xml:space="preserve">FMV growth showing two flat quarters per year.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ACCEPTED with carry-forward labelled on screen. Cadence unchanged.</t>
   </si>
   <si>
     <t xml:space="preserve">D-4</t>
   </si>
   <si>
-    <t xml:space="preserve">Accept the deal-close capture step for round total, NB co-investors and ownership.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Creates ongoing work for his deal leads. Skipping it degrades the leverage KPI silently; coverage monitoring makes the decay visible but the discipline is his.</t>
+    <t xml:space="preserve">Deal-close capture of round total, NB co-investors and ownership.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ACCEPTED. Deal lead completes the capture form at close; coverage monitored on the dashboard.</t>
   </si>
   <si>
     <t xml:space="preserve">D-5</t>
   </si>
   <si>
-    <t xml:space="preserve">Confirm the diversity tile shows coverage and excludes non-reporters, rather than counting unreported as zero.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Changes a mandate figure's meaning. The prototype does not currently distinguish NULL from zero.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">D-6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Confirm which quarter convention each screen displays, now that fiscal and calendar labels differ.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Presentation choice across every quarterly view. Both labels are correct; each screen must state which it uses.</t>
+    <t xml:space="preserve">Diversity tile treatment of non-reporters.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ACCEPTED. Non-reporters excluded from the denominator; coverage shown alongside. NULL never renders as zero.</t>
   </si>
   <si>
     <t xml:space="preserve">A-1</t>
@@ -2660,31 +2663,70 @@
     <t xml:space="preserve">Add women in C-suite and C-suite size to the Visible quarterly request.</t>
   </si>
   <si>
-    <t xml:space="preserve">The diversity mandate tile has no source until this lands. Series begins whenever the request changes.</t>
+    <t xml:space="preserve">The diversity mandate tile has no source until this lands.</t>
   </si>
   <si>
     <t xml:space="preserve">A-2</t>
   </si>
   <si>
-    <t xml:space="preserve">Open the historical backfill workstream: transactions, then rounds, then marks, then ownership.</t>
+    <t xml:space="preserve">Historical backfill: transactions, marks and fund activity. Finance has started.</t>
   </si>
   <si>
     <t xml:space="preserve">CRITICAL PATH. Histories exceed fifteen years for some companies. The app can be built on demo data; it cannot go live without history.</t>
   </si>
   <si>
+    <t xml:space="preserve">Finance + Analyst</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ADR-015</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A-3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Issue the staging templates to Finance and reconcile the first batch against agreed control totals.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Templates issued. Each batch ties to Finance's own control totals before the next begins.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Analyst + Finance</t>
   </si>
   <si>
-    <t xml:space="preserve">ADR-015</t>
-  </si>
-  <si>
-    <t xml:space="preserve">A-3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Draft the Finance transaction upload template and reconcile a first batch.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Phase-1 front door to the registry. Must reject a bad file loudly rather than accept it partially.</t>
+    <t xml:space="preserve">ADR-019</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A-4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Build the company crosswalk: Finance name -&gt; Affinity organisation -&gt; internal company_id.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Must exist BEFORE any transaction loads. Routinely the largest hidden cost in a migration of this kind.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Analyst</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A-5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Establish how far back PER-COMPANY marks exist, as opposed to fund-level NAV only.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">If early history is fund-level only, per-company MOIC and vintage analysis are not reconstructable for those years and the platform must show that boundary.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A-6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Walk D-1 and D-6 through with the VC team lead.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The last two decisions blocking a fully signed-off architecture.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ADR-001, ADR-006</t>
   </si>
   <si>
     <t xml:space="preserve">O-1</t>
@@ -2705,7 +2747,7 @@
     <t xml:space="preserve">Whether the 31 March year end warrants a closer mark.</t>
   </si>
   <si>
-    <t xml:space="preserve">CLOSED: cadence unchanged by this platform. Business as usual for Finance.</t>
+    <t xml:space="preserve">CLOSED: cadence unchanged by this platform.</t>
   </si>
   <si>
     <t xml:space="preserve">O-3</t>
@@ -2718,6 +2760,24 @@
   </si>
   <si>
     <t xml:space="preserve">ADR-017</t>
+  </si>
+  <si>
+    <t xml:space="preserve">O-4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Whether Visible collects the diversity fields.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CLOSED: it does not. Being added to the quarterly request (A-1). NULL, never zero, until the series begins.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">O-5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Whether Visible revenue is run-rate or period actual.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CLOSED: period actual. Resolved into decision D-2.</t>
   </si>
   <si>
     <t xml:space="preserve">O-6</t>
@@ -2900,7 +2960,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="24">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -2965,10 +3025,6 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -3010,7 +3066,7 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="8">
+  <dxfs count="7">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -3054,14 +3110,6 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFE3F2E1"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFF6DC"/>
           <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
@@ -3458,7 +3506,7 @@
       </c>
       <c r="B25" s="8" t="n">
         <f aca="false">COUNTIF('Field Inventory'!M2:M149,"Confirmed")</f>
-        <v>137</v>
+        <v>138</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3476,7 +3524,7 @@
       </c>
       <c r="B27" s="8" t="n">
         <f aca="false">COUNTIF('Field Inventory'!M2:M149,"Open")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6849,7 +6897,7 @@
         <v>376</v>
       </c>
     </row>
-    <row r="73" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="73" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="10" t="s">
         <v>372</v>
       </c>
@@ -6884,8 +6932,8 @@
       <c r="L73" s="10" t="s">
         <v>127</v>
       </c>
-      <c r="M73" s="16" t="s">
-        <v>20</v>
+      <c r="M73" s="12" t="s">
+        <v>16</v>
       </c>
       <c r="N73" s="13" t="s">
         <v>257</v>
@@ -10344,42 +10392,42 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="17" t="s">
+      <c r="A1" s="16" t="s">
         <v>639</v>
       </c>
-      <c r="B1" s="17" t="s">
+      <c r="B1" s="16" t="s">
         <v>640</v>
       </c>
-      <c r="C1" s="17" t="s">
+      <c r="C1" s="16" t="s">
         <v>641</v>
       </c>
-      <c r="D1" s="17" t="s">
+      <c r="D1" s="16" t="s">
         <v>642</v>
       </c>
-      <c r="E1" s="17" t="s">
+      <c r="E1" s="16" t="s">
         <v>643</v>
       </c>
-      <c r="F1" s="17" t="s">
+      <c r="F1" s="16" t="s">
         <v>644</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="18" t="s">
+      <c r="A2" s="17" t="s">
         <v>159</v>
       </c>
-      <c r="B2" s="19" t="s">
+      <c r="B2" s="18" t="s">
         <v>153</v>
       </c>
-      <c r="C2" s="19" t="s">
+      <c r="C2" s="18" t="s">
         <v>49</v>
       </c>
-      <c r="D2" s="19" t="s">
+      <c r="D2" s="18" t="s">
         <v>645</v>
       </c>
-      <c r="E2" s="19" t="s">
+      <c r="E2" s="18" t="s">
         <v>646</v>
       </c>
-      <c r="F2" s="20" t="s">
+      <c r="F2" s="19" t="s">
         <v>647</v>
       </c>
     </row>
@@ -10586,22 +10634,22 @@
       <c r="F15" s="11"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="18" t="s">
+      <c r="A16" s="17" t="s">
         <v>177</v>
       </c>
-      <c r="B16" s="19" t="s">
+      <c r="B16" s="18" t="s">
         <v>667</v>
       </c>
-      <c r="C16" s="19" t="s">
+      <c r="C16" s="18" t="s">
         <v>668</v>
       </c>
-      <c r="D16" s="19" t="s">
+      <c r="D16" s="18" t="s">
         <v>645</v>
       </c>
-      <c r="E16" s="19" t="s">
+      <c r="E16" s="18" t="s">
         <v>646</v>
       </c>
-      <c r="F16" s="20" t="s">
+      <c r="F16" s="19" t="s">
         <v>669</v>
       </c>
     </row>
@@ -10698,22 +10746,22 @@
       <c r="F22" s="11"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="18" t="s">
+      <c r="A23" s="17" t="s">
         <v>142</v>
       </c>
-      <c r="B23" s="19" t="s">
+      <c r="B23" s="18" t="s">
         <v>675</v>
       </c>
-      <c r="C23" s="19" t="s">
+      <c r="C23" s="18" t="s">
         <v>668</v>
       </c>
-      <c r="D23" s="19" t="s">
+      <c r="D23" s="18" t="s">
         <v>645</v>
       </c>
-      <c r="E23" s="19" t="s">
+      <c r="E23" s="18" t="s">
         <v>646</v>
       </c>
-      <c r="F23" s="20" t="s">
+      <c r="F23" s="19" t="s">
         <v>676</v>
       </c>
     </row>
@@ -10912,22 +10960,22 @@
       <c r="F35" s="11"/>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="18" t="s">
+      <c r="A36" s="17" t="s">
         <v>311</v>
       </c>
-      <c r="B36" s="19" t="s">
+      <c r="B36" s="18" t="s">
         <v>684</v>
       </c>
-      <c r="C36" s="19" t="s">
+      <c r="C36" s="18" t="s">
         <v>668</v>
       </c>
-      <c r="D36" s="19" t="s">
+      <c r="D36" s="18" t="s">
         <v>645</v>
       </c>
-      <c r="E36" s="19" t="s">
+      <c r="E36" s="18" t="s">
         <v>646</v>
       </c>
-      <c r="F36" s="20"/>
+      <c r="F36" s="19"/>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="10"/>
@@ -11082,22 +11130,22 @@
       <c r="F46" s="11"/>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="18" t="s">
+      <c r="A47" s="17" t="s">
         <v>703</v>
       </c>
-      <c r="B47" s="19" t="s">
+      <c r="B47" s="18" t="s">
         <v>704</v>
       </c>
-      <c r="C47" s="19" t="s">
+      <c r="C47" s="18" t="s">
         <v>668</v>
       </c>
-      <c r="D47" s="19" t="s">
+      <c r="D47" s="18" t="s">
         <v>645</v>
       </c>
-      <c r="E47" s="19" t="s">
+      <c r="E47" s="18" t="s">
         <v>646</v>
       </c>
-      <c r="F47" s="20" t="s">
+      <c r="F47" s="19" t="s">
         <v>705</v>
       </c>
     </row>
@@ -11180,22 +11228,22 @@
       <c r="F52" s="11"/>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="18" t="s">
+      <c r="A53" s="17" t="s">
         <v>350</v>
       </c>
-      <c r="B53" s="19" t="s">
+      <c r="B53" s="18" t="s">
         <v>710</v>
       </c>
-      <c r="C53" s="19" t="s">
+      <c r="C53" s="18" t="s">
         <v>668</v>
       </c>
-      <c r="D53" s="19" t="s">
+      <c r="D53" s="18" t="s">
         <v>645</v>
       </c>
-      <c r="E53" s="19" t="s">
+      <c r="E53" s="18" t="s">
         <v>646</v>
       </c>
-      <c r="F53" s="20"/>
+      <c r="F53" s="19"/>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="10"/>
@@ -11386,22 +11434,22 @@
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A66" s="18" t="s">
+      <c r="A66" s="17" t="s">
         <v>255</v>
       </c>
-      <c r="B66" s="19" t="s">
+      <c r="B66" s="18" t="s">
         <v>721</v>
       </c>
-      <c r="C66" s="19" t="s">
+      <c r="C66" s="18" t="s">
         <v>668</v>
       </c>
-      <c r="D66" s="19" t="s">
+      <c r="D66" s="18" t="s">
         <v>645</v>
       </c>
-      <c r="E66" s="19" t="s">
+      <c r="E66" s="18" t="s">
         <v>646</v>
       </c>
-      <c r="F66" s="20" t="s">
+      <c r="F66" s="19" t="s">
         <v>722</v>
       </c>
     </row>
@@ -11600,22 +11648,22 @@
       <c r="F79" s="11"/>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A80" s="18" t="s">
+      <c r="A80" s="17" t="s">
         <v>193</v>
       </c>
-      <c r="B80" s="19" t="s">
+      <c r="B80" s="18" t="s">
         <v>732</v>
       </c>
-      <c r="C80" s="19" t="s">
+      <c r="C80" s="18" t="s">
         <v>668</v>
       </c>
-      <c r="D80" s="19" t="s">
+      <c r="D80" s="18" t="s">
         <v>645</v>
       </c>
-      <c r="E80" s="19" t="s">
+      <c r="E80" s="18" t="s">
         <v>646</v>
       </c>
-      <c r="F80" s="20" t="s">
+      <c r="F80" s="19" t="s">
         <v>733</v>
       </c>
     </row>
@@ -11694,22 +11742,22 @@
       </c>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A86" s="18" t="s">
+      <c r="A86" s="17" t="s">
         <v>438</v>
       </c>
-      <c r="B86" s="19" t="s">
+      <c r="B86" s="18" t="s">
         <v>439</v>
       </c>
-      <c r="C86" s="19" t="s">
+      <c r="C86" s="18" t="s">
         <v>49</v>
       </c>
-      <c r="D86" s="19" t="s">
+      <c r="D86" s="18" t="s">
         <v>645</v>
       </c>
-      <c r="E86" s="19" t="s">
+      <c r="E86" s="18" t="s">
         <v>646</v>
       </c>
-      <c r="F86" s="20" t="s">
+      <c r="F86" s="19" t="s">
         <v>736</v>
       </c>
     </row>
@@ -11868,22 +11916,22 @@
       <c r="F97" s="11"/>
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A98" s="18" t="s">
+      <c r="A98" s="17" t="s">
         <v>459</v>
       </c>
-      <c r="B98" s="19" t="s">
+      <c r="B98" s="18" t="s">
         <v>737</v>
       </c>
-      <c r="C98" s="19" t="s">
+      <c r="C98" s="18" t="s">
         <v>668</v>
       </c>
-      <c r="D98" s="19" t="s">
+      <c r="D98" s="18" t="s">
         <v>645</v>
       </c>
-      <c r="E98" s="19" t="s">
+      <c r="E98" s="18" t="s">
         <v>646</v>
       </c>
-      <c r="F98" s="20" t="s">
+      <c r="F98" s="19" t="s">
         <v>738</v>
       </c>
     </row>
@@ -11948,22 +11996,22 @@
       </c>
     </row>
     <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A103" s="18" t="s">
+      <c r="A103" s="17" t="s">
         <v>45</v>
       </c>
-      <c r="B103" s="19" t="s">
+      <c r="B103" s="18" t="s">
         <v>741</v>
       </c>
-      <c r="C103" s="19" t="s">
+      <c r="C103" s="18" t="s">
         <v>628</v>
       </c>
-      <c r="D103" s="19" t="s">
+      <c r="D103" s="18" t="s">
         <v>645</v>
       </c>
-      <c r="E103" s="19" t="s">
+      <c r="E103" s="18" t="s">
         <v>646</v>
       </c>
-      <c r="F103" s="20" t="s">
+      <c r="F103" s="19" t="s">
         <v>742</v>
       </c>
     </row>
@@ -12158,22 +12206,22 @@
       </c>
     </row>
     <row r="117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A117" s="18" t="s">
+      <c r="A117" s="17" t="s">
         <v>125</v>
       </c>
-      <c r="B117" s="19" t="s">
+      <c r="B117" s="18" t="s">
         <v>747</v>
       </c>
-      <c r="C117" s="19" t="s">
+      <c r="C117" s="18" t="s">
         <v>668</v>
       </c>
-      <c r="D117" s="19" t="s">
+      <c r="D117" s="18" t="s">
         <v>645</v>
       </c>
-      <c r="E117" s="19" t="s">
+      <c r="E117" s="18" t="s">
         <v>646</v>
       </c>
-      <c r="F117" s="20" t="s">
+      <c r="F117" s="19" t="s">
         <v>748</v>
       </c>
     </row>
@@ -12270,22 +12318,22 @@
       </c>
     </row>
     <row r="124" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A124" s="18" t="s">
+      <c r="A124" s="17" t="s">
         <v>502</v>
       </c>
-      <c r="B124" s="19" t="s">
+      <c r="B124" s="18" t="s">
         <v>503</v>
       </c>
-      <c r="C124" s="19" t="s">
+      <c r="C124" s="18" t="s">
         <v>49</v>
       </c>
-      <c r="D124" s="19" t="s">
+      <c r="D124" s="18" t="s">
         <v>645</v>
       </c>
-      <c r="E124" s="19" t="s">
+      <c r="E124" s="18" t="s">
         <v>646</v>
       </c>
-      <c r="F124" s="20" t="s">
+      <c r="F124" s="19" t="s">
         <v>754</v>
       </c>
     </row>
@@ -12506,22 +12554,22 @@
       </c>
     </row>
     <row r="139" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A139" s="18" t="s">
+      <c r="A139" s="17" t="s">
         <v>540</v>
       </c>
-      <c r="B139" s="19" t="s">
+      <c r="B139" s="18" t="s">
         <v>763</v>
       </c>
-      <c r="C139" s="19" t="s">
+      <c r="C139" s="18" t="s">
         <v>668</v>
       </c>
-      <c r="D139" s="19" t="s">
+      <c r="D139" s="18" t="s">
         <v>645</v>
       </c>
-      <c r="E139" s="19" t="s">
+      <c r="E139" s="18" t="s">
         <v>646</v>
       </c>
-      <c r="F139" s="20"/>
+      <c r="F139" s="19"/>
     </row>
     <row r="140" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A140" s="10"/>
@@ -12614,22 +12662,22 @@
       <c r="F145" s="11"/>
     </row>
     <row r="146" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A146" s="18" t="s">
+      <c r="A146" s="17" t="s">
         <v>579</v>
       </c>
-      <c r="B146" s="19" t="s">
+      <c r="B146" s="18" t="s">
         <v>769</v>
       </c>
-      <c r="C146" s="19" t="s">
+      <c r="C146" s="18" t="s">
         <v>668</v>
       </c>
-      <c r="D146" s="19" t="s">
+      <c r="D146" s="18" t="s">
         <v>645</v>
       </c>
-      <c r="E146" s="19" t="s">
+      <c r="E146" s="18" t="s">
         <v>646</v>
       </c>
-      <c r="F146" s="20" t="s">
+      <c r="F146" s="19" t="s">
         <v>770</v>
       </c>
     </row>
@@ -12754,22 +12802,22 @@
       <c r="F154" s="11"/>
     </row>
     <row r="155" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A155" s="18" t="s">
+      <c r="A155" s="17" t="s">
         <v>592</v>
       </c>
-      <c r="B155" s="19" t="s">
+      <c r="B155" s="18" t="s">
         <v>778</v>
       </c>
-      <c r="C155" s="19" t="s">
+      <c r="C155" s="18" t="s">
         <v>668</v>
       </c>
-      <c r="D155" s="19" t="s">
+      <c r="D155" s="18" t="s">
         <v>645</v>
       </c>
-      <c r="E155" s="19" t="s">
+      <c r="E155" s="18" t="s">
         <v>646</v>
       </c>
-      <c r="F155" s="20"/>
+      <c r="F155" s="19"/>
     </row>
     <row r="156" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A156" s="10"/>
@@ -12836,22 +12884,22 @@
       </c>
     </row>
     <row r="160" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A160" s="18" t="s">
+      <c r="A160" s="17" t="s">
         <v>785</v>
       </c>
-      <c r="B160" s="19" t="s">
+      <c r="B160" s="18" t="s">
         <v>786</v>
       </c>
-      <c r="C160" s="19" t="s">
+      <c r="C160" s="18" t="s">
         <v>668</v>
       </c>
-      <c r="D160" s="19" t="s">
+      <c r="D160" s="18" t="s">
         <v>645</v>
       </c>
-      <c r="E160" s="19" t="s">
+      <c r="E160" s="18" t="s">
         <v>646</v>
       </c>
-      <c r="F160" s="20" t="s">
+      <c r="F160" s="19" t="s">
         <v>787</v>
       </c>
     </row>
@@ -12958,22 +13006,22 @@
       <c r="F167" s="11"/>
     </row>
     <row r="168" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A168" s="18" t="s">
+      <c r="A168" s="17" t="s">
         <v>795</v>
       </c>
-      <c r="B168" s="19" t="s">
+      <c r="B168" s="18" t="s">
         <v>796</v>
       </c>
-      <c r="C168" s="19" t="s">
+      <c r="C168" s="18" t="s">
         <v>665</v>
       </c>
-      <c r="D168" s="19" t="s">
+      <c r="D168" s="18" t="s">
         <v>645</v>
       </c>
-      <c r="E168" s="19" t="s">
+      <c r="E168" s="18" t="s">
         <v>646</v>
       </c>
-      <c r="F168" s="20" t="s">
+      <c r="F168" s="19" t="s">
         <v>797</v>
       </c>
     </row>
@@ -13152,7 +13200,7 @@
       <c r="A4" s="11" t="s">
         <v>79</v>
       </c>
-      <c r="B4" s="21" t="s">
+      <c r="B4" s="20" t="s">
         <v>817</v>
       </c>
       <c r="C4" s="11" t="s">
@@ -13198,7 +13246,7 @@
       <c r="A6" s="11" t="s">
         <v>243</v>
       </c>
-      <c r="B6" s="21" t="s">
+      <c r="B6" s="20" t="s">
         <v>826</v>
       </c>
       <c r="C6" s="11" t="s">
@@ -13267,7 +13315,7 @@
       <c r="A9" s="11" t="s">
         <v>50</v>
       </c>
-      <c r="B9" s="21" t="s">
+      <c r="B9" s="20" t="s">
         <v>840</v>
       </c>
       <c r="C9" s="11" t="s">
@@ -13325,7 +13373,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:F19"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="8"/>
@@ -13337,27 +13385,27 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="17" t="s">
+      <c r="A1" s="16" t="s">
         <v>850</v>
       </c>
-      <c r="B1" s="17" t="s">
+      <c r="B1" s="16" t="s">
         <v>33</v>
       </c>
-      <c r="C1" s="17" t="s">
+      <c r="C1" s="16" t="s">
         <v>851</v>
       </c>
-      <c r="D1" s="17" t="s">
+      <c r="D1" s="16" t="s">
         <v>852</v>
       </c>
-      <c r="E1" s="17" t="s">
+      <c r="E1" s="16" t="s">
         <v>807</v>
       </c>
-      <c r="F1" s="17" t="s">
+      <c r="F1" s="16" t="s">
         <v>853</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="22" t="s">
+      <c r="A2" s="21" t="s">
         <v>854</v>
       </c>
       <c r="B2" s="11" t="s">
@@ -13372,12 +13420,12 @@
       <c r="E2" s="11" t="s">
         <v>858</v>
       </c>
-      <c r="F2" s="23" t="s">
+      <c r="F2" s="22" t="s">
         <v>586</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="22" t="s">
+    <row r="3" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="21" t="s">
         <v>859</v>
       </c>
       <c r="B3" s="11" t="s">
@@ -13392,228 +13440,328 @@
       <c r="E3" s="11" t="s">
         <v>858</v>
       </c>
-      <c r="F3" s="23" t="s">
-        <v>53</v>
+      <c r="F3" s="22" t="s">
+        <v>128</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="22" t="s">
+      <c r="A4" s="23" t="s">
         <v>862</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>855</v>
+        <v>863</v>
       </c>
       <c r="C4" s="11" t="s">
-        <v>863</v>
+        <v>864</v>
       </c>
       <c r="D4" s="11" t="s">
-        <v>864</v>
+        <v>865</v>
       </c>
       <c r="E4" s="11" t="s">
         <v>858</v>
       </c>
-      <c r="F4" s="23" t="s">
-        <v>353</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="22" t="s">
-        <v>865</v>
+      <c r="F4" s="22" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="23" t="s">
+        <v>866</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>855</v>
+        <v>863</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>866</v>
+        <v>867</v>
       </c>
       <c r="D5" s="11" t="s">
-        <v>867</v>
+        <v>868</v>
       </c>
       <c r="E5" s="11" t="s">
         <v>858</v>
       </c>
-      <c r="F5" s="23" t="s">
-        <v>196</v>
+      <c r="F5" s="22" t="s">
+        <v>353</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="22" t="s">
-        <v>868</v>
+      <c r="A6" s="23" t="s">
+        <v>869</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>855</v>
+        <v>863</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>869</v>
+        <v>870</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>870</v>
+        <v>871</v>
       </c>
       <c r="E6" s="11" t="s">
         <v>858</v>
       </c>
-      <c r="F6" s="23" t="s">
-        <v>257</v>
+      <c r="F6" s="22" t="s">
+        <v>196</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="22" t="s">
-        <v>871</v>
+      <c r="A7" s="23" t="s">
+        <v>872</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>855</v>
+        <v>863</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>872</v>
+        <v>873</v>
       </c>
       <c r="D7" s="11" t="s">
-        <v>873</v>
+        <v>874</v>
       </c>
       <c r="E7" s="11" t="s">
         <v>858</v>
       </c>
-      <c r="F7" s="23" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="21" t="s">
-        <v>874</v>
+      <c r="F7" s="22" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="20" t="s">
+        <v>875</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>875</v>
+        <v>876</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>876</v>
+        <v>877</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>877</v>
+        <v>878</v>
       </c>
       <c r="E8" s="11" t="s">
         <v>812</v>
       </c>
-      <c r="F8" s="23" t="s">
+      <c r="F8" s="22" t="s">
         <v>257</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="21" t="s">
-        <v>878</v>
+      <c r="A9" s="20" t="s">
+        <v>879</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>875</v>
+        <v>876</v>
       </c>
       <c r="C9" s="11" t="s">
-        <v>879</v>
+        <v>880</v>
       </c>
       <c r="D9" s="11" t="s">
-        <v>880</v>
+        <v>881</v>
       </c>
       <c r="E9" s="11" t="s">
-        <v>881</v>
-      </c>
-      <c r="F9" s="23" t="s">
         <v>882</v>
       </c>
+      <c r="F9" s="22" t="s">
+        <v>883</v>
+      </c>
     </row>
     <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="21" t="s">
-        <v>883</v>
+      <c r="A10" s="20" t="s">
+        <v>884</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>875</v>
+        <v>876</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>884</v>
+        <v>885</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>885</v>
+        <v>886</v>
       </c>
       <c r="E10" s="11" t="s">
-        <v>881</v>
-      </c>
-      <c r="F10" s="23" t="s">
-        <v>82</v>
+        <v>887</v>
+      </c>
+      <c r="F10" s="22" t="s">
+        <v>888</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="24" t="s">
-        <v>886</v>
+      <c r="A11" s="20" t="s">
+        <v>889</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>887</v>
+        <v>876</v>
       </c>
       <c r="C11" s="11" t="s">
+        <v>890</v>
+      </c>
+      <c r="D11" s="11" t="s">
+        <v>891</v>
+      </c>
+      <c r="E11" s="11" t="s">
+        <v>892</v>
+      </c>
+      <c r="F11" s="22" t="s">
         <v>888</v>
       </c>
-      <c r="D11" s="11" t="s">
-        <v>889</v>
-      </c>
-      <c r="E11" s="11" t="s">
-        <v>113</v>
-      </c>
-      <c r="F11" s="23" t="s">
-        <v>353</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="24" t="s">
-        <v>890</v>
+    </row>
+    <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="20" t="s">
+        <v>893</v>
       </c>
       <c r="B12" s="11" t="s">
-        <v>887</v>
+        <v>876</v>
       </c>
       <c r="C12" s="11" t="s">
-        <v>891</v>
+        <v>894</v>
       </c>
       <c r="D12" s="11" t="s">
+        <v>895</v>
+      </c>
+      <c r="E12" s="11" t="s">
+        <v>80</v>
+      </c>
+      <c r="F12" s="22" t="s">
+        <v>888</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="20" t="s">
+        <v>896</v>
+      </c>
+      <c r="B13" s="11" t="s">
+        <v>876</v>
+      </c>
+      <c r="C13" s="11" t="s">
+        <v>897</v>
+      </c>
+      <c r="D13" s="11" t="s">
+        <v>898</v>
+      </c>
+      <c r="E13" s="11" t="s">
         <v>892</v>
       </c>
-      <c r="E12" s="11" t="s">
-        <v>113</v>
-      </c>
-      <c r="F12" s="23" t="s">
-        <v>353</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="24" t="s">
-        <v>893</v>
-      </c>
-      <c r="B13" s="11" t="s">
-        <v>887</v>
-      </c>
-      <c r="C13" s="11" t="s">
-        <v>894</v>
-      </c>
-      <c r="D13" s="11" t="s">
-        <v>895</v>
-      </c>
-      <c r="E13" s="11" t="s">
-        <v>113</v>
-      </c>
-      <c r="F13" s="23" t="s">
-        <v>896</v>
+      <c r="F13" s="22" t="s">
+        <v>899</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="24" t="s">
-        <v>897</v>
+      <c r="A14" s="23" t="s">
+        <v>900</v>
       </c>
       <c r="B14" s="11" t="s">
-        <v>887</v>
+        <v>901</v>
       </c>
       <c r="C14" s="11" t="s">
-        <v>898</v>
+        <v>902</v>
       </c>
       <c r="D14" s="11" t="s">
-        <v>899</v>
+        <v>903</v>
       </c>
       <c r="E14" s="11" t="s">
         <v>113</v>
       </c>
-      <c r="F14" s="23" t="s">
-        <v>882</v>
+      <c r="F14" s="22" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="23" t="s">
+        <v>904</v>
+      </c>
+      <c r="B15" s="11" t="s">
+        <v>901</v>
+      </c>
+      <c r="C15" s="11" t="s">
+        <v>905</v>
+      </c>
+      <c r="D15" s="11" t="s">
+        <v>906</v>
+      </c>
+      <c r="E15" s="11" t="s">
+        <v>113</v>
+      </c>
+      <c r="F15" s="22" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="23" t="s">
+        <v>907</v>
+      </c>
+      <c r="B16" s="11" t="s">
+        <v>901</v>
+      </c>
+      <c r="C16" s="11" t="s">
+        <v>908</v>
+      </c>
+      <c r="D16" s="11" t="s">
+        <v>909</v>
+      </c>
+      <c r="E16" s="11" t="s">
+        <v>113</v>
+      </c>
+      <c r="F16" s="22" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="23" t="s">
+        <v>911</v>
+      </c>
+      <c r="B17" s="11" t="s">
+        <v>901</v>
+      </c>
+      <c r="C17" s="11" t="s">
+        <v>912</v>
+      </c>
+      <c r="D17" s="11" t="s">
+        <v>913</v>
+      </c>
+      <c r="E17" s="11" t="s">
+        <v>113</v>
+      </c>
+      <c r="F17" s="22" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="23" t="s">
+        <v>914</v>
+      </c>
+      <c r="B18" s="11" t="s">
+        <v>901</v>
+      </c>
+      <c r="C18" s="11" t="s">
+        <v>915</v>
+      </c>
+      <c r="D18" s="11" t="s">
+        <v>916</v>
+      </c>
+      <c r="E18" s="11" t="s">
+        <v>113</v>
+      </c>
+      <c r="F18" s="22" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="23" t="s">
+        <v>917</v>
+      </c>
+      <c r="B19" s="11" t="s">
+        <v>901</v>
+      </c>
+      <c r="C19" s="11" t="s">
+        <v>918</v>
+      </c>
+      <c r="D19" s="11" t="s">
+        <v>919</v>
+      </c>
+      <c r="E19" s="11" t="s">
+        <v>113</v>
+      </c>
+      <c r="F19" s="22" t="s">
+        <v>883</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Finalized architecture, added delivery roadmap
</commit_message>
<xml_diff>
--- a/portfolio-command-field-inventory.xlsx
+++ b/portfolio-command-field-inventory.xlsx
@@ -27,12 +27,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2985" uniqueCount="920">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2991" uniqueCount="923">
   <si>
     <t xml:space="preserve">Portfolio Command - Master Data Field Inventory</t>
   </si>
   <si>
-    <t xml:space="preserve">Rev 4 - 28 July 2026. All twelve questions and all six open items closed. Two decisions outstanding with the VC team lead: D-1 and D-6.</t>
+    <t xml:space="preserve">Rev 5 - 28 July 2026. All questions, open items and decisions closed. Architecture and data design signed off; build sequence in delivery-roadmap.md.</t>
   </si>
   <si>
     <t xml:space="preserve">What changed in this revision</t>
@@ -92,7 +92,7 @@
     <t xml:space="preserve">Open</t>
   </si>
   <si>
-    <t xml:space="preserve">Outstanding decision. Only D-1 and D-6 remain, both with the VC team lead.</t>
+    <t xml:space="preserve">No rows remain in this state - all decisions are settled as of 28 July 2026.</t>
   </si>
   <si>
     <t xml:space="preserve">Field counts (live formulas)</t>
@@ -2594,13 +2594,13 @@
     <t xml:space="preserve">D-1</t>
   </si>
   <si>
-    <t xml:space="preserve">OUTSTANDING</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Confirm the import contract may treat derived fields as advisory, correcting them against the transactions and returning a reconciliation warning.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Still to be walked through with Daniel. His stated requirement was that the contract stay intact; this is the one place his workflow behaviour changes.</t>
+    <t xml:space="preserve">Settled</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Import contract may treat derived fields as advisory.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ACCEPTED. Import corrects against the transactions and returns a reconciliation warning rather than accepting a contradicting figure.</t>
   </si>
   <si>
     <t xml:space="preserve">Daniel Armali</t>
@@ -2609,18 +2609,15 @@
     <t xml:space="preserve">D-6</t>
   </si>
   <si>
-    <t xml:space="preserve">Confirm which quarter convention each screen displays, now that fiscal and calendar labels differ.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Still to be walked through with Daniel. Suggested split: fiscal on Reports and board-facing views, calendar on the Portfolio KPI history.</t>
+    <t xml:space="preserve">Quarter convention per screen.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ACCEPTED. Fiscal labels on Reports and board-facing views; calendar labels on the Portfolio KPI history. Every view states which it uses.</t>
   </si>
   <si>
     <t xml:space="preserve">D-2</t>
   </si>
   <si>
-    <t xml:space="preserve">Settled</t>
-  </si>
-  <si>
     <t xml:space="preserve">How revenue is presented.</t>
   </si>
   <si>
@@ -2720,19 +2717,31 @@
     <t xml:space="preserve">A-6</t>
   </si>
   <si>
+    <t xml:space="preserve">Closed</t>
+  </si>
+  <si>
     <t xml:space="preserve">Walk D-1 and D-6 through with the VC team lead.</t>
   </si>
   <si>
-    <t xml:space="preserve">The last two decisions blocking a fully signed-off architecture.</t>
+    <t xml:space="preserve">COMPLETE 28 Jul 2026. All architecture and data decisions are now signed off.</t>
   </si>
   <si>
     <t xml:space="preserve">ADR-001, ADR-006</t>
   </si>
   <si>
+    <t xml:space="preserve">A-7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Confirm Affinity v2 and Visible.vc API access on current plan tiers.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Both are assumed by the ingestion design. Plan-tier restrictions are cheap to discover now and expensive to discover mid-build.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ADR-009, ADR-010</t>
+  </si>
+  <si>
     <t xml:space="preserve">O-1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Closed</t>
   </si>
   <si>
     <t xml:space="preserve">Valuation effective date vs data cutoff.</t>
@@ -2960,7 +2969,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="23">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -3045,15 +3054,11 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -13373,7 +13378,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F19"/>
+  <dimension ref="A1:F20"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="8"/>
@@ -13445,17 +13450,17 @@
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="23" t="s">
+      <c r="A4" s="21" t="s">
         <v>862</v>
       </c>
       <c r="B4" s="11" t="s">
+        <v>855</v>
+      </c>
+      <c r="C4" s="11" t="s">
         <v>863</v>
       </c>
-      <c r="C4" s="11" t="s">
+      <c r="D4" s="11" t="s">
         <v>864</v>
-      </c>
-      <c r="D4" s="11" t="s">
-        <v>865</v>
       </c>
       <c r="E4" s="11" t="s">
         <v>858</v>
@@ -13465,17 +13470,17 @@
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="23" t="s">
+      <c r="A5" s="21" t="s">
+        <v>865</v>
+      </c>
+      <c r="B5" s="11" t="s">
+        <v>855</v>
+      </c>
+      <c r="C5" s="11" t="s">
         <v>866</v>
       </c>
-      <c r="B5" s="11" t="s">
-        <v>863</v>
-      </c>
-      <c r="C5" s="11" t="s">
+      <c r="D5" s="11" t="s">
         <v>867</v>
-      </c>
-      <c r="D5" s="11" t="s">
-        <v>868</v>
       </c>
       <c r="E5" s="11" t="s">
         <v>858</v>
@@ -13485,17 +13490,17 @@
       </c>
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="23" t="s">
+      <c r="A6" s="21" t="s">
+        <v>868</v>
+      </c>
+      <c r="B6" s="11" t="s">
+        <v>855</v>
+      </c>
+      <c r="C6" s="11" t="s">
         <v>869</v>
       </c>
-      <c r="B6" s="11" t="s">
-        <v>863</v>
-      </c>
-      <c r="C6" s="11" t="s">
+      <c r="D6" s="11" t="s">
         <v>870</v>
-      </c>
-      <c r="D6" s="11" t="s">
-        <v>871</v>
       </c>
       <c r="E6" s="11" t="s">
         <v>858</v>
@@ -13505,17 +13510,17 @@
       </c>
     </row>
     <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="23" t="s">
+      <c r="A7" s="21" t="s">
+        <v>871</v>
+      </c>
+      <c r="B7" s="11" t="s">
+        <v>855</v>
+      </c>
+      <c r="C7" s="11" t="s">
         <v>872</v>
       </c>
-      <c r="B7" s="11" t="s">
-        <v>863</v>
-      </c>
-      <c r="C7" s="11" t="s">
+      <c r="D7" s="11" t="s">
         <v>873</v>
-      </c>
-      <c r="D7" s="11" t="s">
-        <v>874</v>
       </c>
       <c r="E7" s="11" t="s">
         <v>858</v>
@@ -13526,16 +13531,16 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="20" t="s">
+        <v>874</v>
+      </c>
+      <c r="B8" s="11" t="s">
         <v>875</v>
       </c>
-      <c r="B8" s="11" t="s">
+      <c r="C8" s="11" t="s">
         <v>876</v>
       </c>
-      <c r="C8" s="11" t="s">
+      <c r="D8" s="11" t="s">
         <v>877</v>
-      </c>
-      <c r="D8" s="11" t="s">
-        <v>878</v>
       </c>
       <c r="E8" s="11" t="s">
         <v>812</v>
@@ -13546,90 +13551,90 @@
     </row>
     <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="20" t="s">
+        <v>878</v>
+      </c>
+      <c r="B9" s="11" t="s">
+        <v>875</v>
+      </c>
+      <c r="C9" s="11" t="s">
         <v>879</v>
       </c>
-      <c r="B9" s="11" t="s">
-        <v>876</v>
-      </c>
-      <c r="C9" s="11" t="s">
+      <c r="D9" s="11" t="s">
         <v>880</v>
       </c>
-      <c r="D9" s="11" t="s">
+      <c r="E9" s="11" t="s">
         <v>881</v>
       </c>
-      <c r="E9" s="11" t="s">
+      <c r="F9" s="22" t="s">
         <v>882</v>
-      </c>
-      <c r="F9" s="22" t="s">
-        <v>883</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="20" t="s">
+        <v>883</v>
+      </c>
+      <c r="B10" s="11" t="s">
+        <v>875</v>
+      </c>
+      <c r="C10" s="11" t="s">
         <v>884</v>
       </c>
-      <c r="B10" s="11" t="s">
-        <v>876</v>
-      </c>
-      <c r="C10" s="11" t="s">
+      <c r="D10" s="11" t="s">
         <v>885</v>
       </c>
-      <c r="D10" s="11" t="s">
+      <c r="E10" s="11" t="s">
         <v>886</v>
       </c>
-      <c r="E10" s="11" t="s">
+      <c r="F10" s="22" t="s">
         <v>887</v>
-      </c>
-      <c r="F10" s="22" t="s">
-        <v>888</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="20" t="s">
+        <v>888</v>
+      </c>
+      <c r="B11" s="11" t="s">
+        <v>875</v>
+      </c>
+      <c r="C11" s="11" t="s">
         <v>889</v>
       </c>
-      <c r="B11" s="11" t="s">
-        <v>876</v>
-      </c>
-      <c r="C11" s="11" t="s">
+      <c r="D11" s="11" t="s">
         <v>890</v>
       </c>
-      <c r="D11" s="11" t="s">
+      <c r="E11" s="11" t="s">
         <v>891</v>
       </c>
-      <c r="E11" s="11" t="s">
-        <v>892</v>
-      </c>
       <c r="F11" s="22" t="s">
-        <v>888</v>
+        <v>887</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="20" t="s">
+        <v>892</v>
+      </c>
+      <c r="B12" s="11" t="s">
+        <v>875</v>
+      </c>
+      <c r="C12" s="11" t="s">
         <v>893</v>
       </c>
-      <c r="B12" s="11" t="s">
-        <v>876</v>
-      </c>
-      <c r="C12" s="11" t="s">
+      <c r="D12" s="11" t="s">
         <v>894</v>
-      </c>
-      <c r="D12" s="11" t="s">
-        <v>895</v>
       </c>
       <c r="E12" s="11" t="s">
         <v>80</v>
       </c>
       <c r="F12" s="22" t="s">
-        <v>888</v>
+        <v>887</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="20" t="s">
+      <c r="A13" s="21" t="s">
+        <v>895</v>
+      </c>
+      <c r="B13" s="11" t="s">
         <v>896</v>
-      </c>
-      <c r="B13" s="11" t="s">
-        <v>876</v>
       </c>
       <c r="C13" s="11" t="s">
         <v>897</v>
@@ -13638,38 +13643,38 @@
         <v>898</v>
       </c>
       <c r="E13" s="11" t="s">
-        <v>892</v>
+        <v>891</v>
       </c>
       <c r="F13" s="22" t="s">
         <v>899</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="23" t="s">
+      <c r="A14" s="20" t="s">
         <v>900</v>
       </c>
       <c r="B14" s="11" t="s">
+        <v>875</v>
+      </c>
+      <c r="C14" s="11" t="s">
         <v>901</v>
       </c>
-      <c r="C14" s="11" t="s">
+      <c r="D14" s="11" t="s">
         <v>902</v>
       </c>
-      <c r="D14" s="11" t="s">
+      <c r="E14" s="11" t="s">
+        <v>891</v>
+      </c>
+      <c r="F14" s="22" t="s">
         <v>903</v>
       </c>
-      <c r="E14" s="11" t="s">
-        <v>113</v>
-      </c>
-      <c r="F14" s="22" t="s">
-        <v>353</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="23" t="s">
+    </row>
+    <row r="15" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="21" t="s">
         <v>904</v>
       </c>
       <c r="B15" s="11" t="s">
-        <v>901</v>
+        <v>896</v>
       </c>
       <c r="C15" s="11" t="s">
         <v>905</v>
@@ -13684,12 +13689,12 @@
         <v>353</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="23" t="s">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="21" t="s">
         <v>907</v>
       </c>
       <c r="B16" s="11" t="s">
-        <v>901</v>
+        <v>896</v>
       </c>
       <c r="C16" s="11" t="s">
         <v>908</v>
@@ -13701,35 +13706,35 @@
         <v>113</v>
       </c>
       <c r="F16" s="22" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="21" t="s">
         <v>910</v>
       </c>
-    </row>
-    <row r="17" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="23" t="s">
+      <c r="B17" s="11" t="s">
+        <v>896</v>
+      </c>
+      <c r="C17" s="11" t="s">
         <v>911</v>
       </c>
-      <c r="B17" s="11" t="s">
-        <v>901</v>
-      </c>
-      <c r="C17" s="11" t="s">
+      <c r="D17" s="11" t="s">
         <v>912</v>
-      </c>
-      <c r="D17" s="11" t="s">
-        <v>913</v>
       </c>
       <c r="E17" s="11" t="s">
         <v>113</v>
       </c>
       <c r="F17" s="22" t="s">
-        <v>257</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="23" t="s">
+        <v>913</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="21" t="s">
         <v>914</v>
       </c>
       <c r="B18" s="11" t="s">
-        <v>901</v>
+        <v>896</v>
       </c>
       <c r="C18" s="11" t="s">
         <v>915</v>
@@ -13741,15 +13746,15 @@
         <v>113</v>
       </c>
       <c r="F18" s="22" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="23" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="21" t="s">
         <v>917</v>
       </c>
       <c r="B19" s="11" t="s">
-        <v>901</v>
+        <v>896</v>
       </c>
       <c r="C19" s="11" t="s">
         <v>918</v>
@@ -13761,7 +13766,27 @@
         <v>113</v>
       </c>
       <c r="F19" s="22" t="s">
-        <v>883</v>
+        <v>53</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="21" t="s">
+        <v>920</v>
+      </c>
+      <c r="B20" s="11" t="s">
+        <v>896</v>
+      </c>
+      <c r="C20" s="11" t="s">
+        <v>921</v>
+      </c>
+      <c r="D20" s="11" t="s">
+        <v>922</v>
+      </c>
+      <c r="E20" s="11" t="s">
+        <v>113</v>
+      </c>
+      <c r="F20" s="22" t="s">
+        <v>882</v>
       </c>
     </row>
   </sheetData>

</xml_diff>